<commit_message>
T1: datasets, Introduction v3, deconvolution method readings and selection, ADEMP draft update
</commit_message>
<xml_diff>
--- a/thesis/data_inventory.xlsx
+++ b/thesis/data_inventory.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1808" yWindow="1808" windowWidth="17279" windowHeight="9982" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-3240" yWindow="-21710" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="inventory" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,10 +31,26 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -43,7 +59,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDDDDD"/>
+        <fgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.3999755851924192"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9EC9F"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -71,79 +99,34 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -436,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2968,6 +2951,252 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>CRC across the age continuum (snRNA atlas, GEO 2026)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GEO GSE312983 (no PubMed ID on GEO yet)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE312983</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>189 (one primary tumour per patient, obs FRID)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>850222</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>52 (Annotation_Tier2; 7 in Tier1)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>10x 3' (snRNA, nuclei; version TO VERIFY)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>colorectal cancer (tumour only, no normal)</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>not on CELLxGENE</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>GEO submitted 2025-12-09, public 2026-09-23</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>GEO public; FASTQ controlled (dbGaP)</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>alternative colon dataset (training/held-out/E' by donor)</t>
+        </is>
+      </c>
+      <c r="O33" s="9" t="inlineStr">
+        <is>
+          <t>RAW COUNTS ONLY FOR 4,070 HVGs (layers/counts); all 36,601 genes only log-normalised (raw/X). h5ad 54 GB; obs has Age, Sex, Site, MSI, Stage, Therapy. Unsorted, all compartments. Nuclei, unlike Pelka cells.</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Lee 2020 SMC (CRC + matched normal)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>doi:10.1038/s41588-020-0636-z (PMID 32451460)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE132465</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>23 (10 with matched normal)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>63689</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>TO VERIFY (Cell_type + Cell_subtype columns)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>10x 3' (version TO VERIFY, probably v2)</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>colorectal cancer; normal mucosa</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>not on CELLxGENE</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>GEO public 2020-04-04</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>GEO public</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>alternative colon dataset (training/held-out/E' by donor)</t>
+        </is>
+      </c>
+      <c r="O34" s="11" t="inlineStr">
+        <is>
+          <t>PREFERRED over GSE166555 (Claude, 2026-10-23): meets every rule; one raw UMI matrix with all genes; per-cell patient, tumour/normal, cell type and subtype. Files: raw_UMI_count_matrix.txt.gz + cell_annotation.txt.gz.</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Uhlitz 2021 (CRC + normal)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>doi:10.15252/emmm.202114123 (EMBO Mol Med 2021; PMID 34409732)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE166555</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>~68700</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>TO VERIFY (per compartment)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>10x 3' v2</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>colorectal cancer; normal</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>not on CELLxGENE</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>GEO public 2021-02-11</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>GEO public</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>alternative colon dataset (second choice)</t>
+        </is>
+      </c>
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t>Second choice after GSE132465: only 12 donors (just above the minimum of 10); raw counts only per sample inside GSE166555_RAW.tar; labels split by compartment (epi/imm/str).</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2979,21 +3208,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:O24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="6" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="9" max="10"/>
+    <col width="14" customWidth="1" min="11" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
@@ -3023,7 +3249,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3. Lymphoid: 10x 3' only. Colon: healthy or CRC only (no IBD). Brain: single-nucleus accepted (no healthy adult whole-cell brain data exist).</t>
+          <t>3. Lymphoid: 10x 5' accepted (changed 2026-10-23: comparisons are within tissue; was 3' only). Colon: healthy or CRC only (no IBD), paired tumour + normal per donor preferred. Brain: single-nucleus accepted (no healthy adult whole-cell brain data exist).</t>
         </is>
       </c>
     </row>
@@ -3034,14 +3260,9 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5. OPEN: keep E' (as donor-variability benchmark, reword PROTOCOLLO 5.6) or drop it. OPEN: arm G only where data are post-cutoff.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8" ht="28.5" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>status</t>
@@ -3118,84 +3339,84 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="9" ht="42.75" customFormat="1" customHeight="1" s="6">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>training + held-out + E' (by donor)</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>brain (DLPFC)</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>normal adults</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>PsychAD 2024, doi:10.1101/2024.10.31.24316513</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>preprint 2024-10-31; CELLxGENE 2025-07-29</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>10x 3' v3</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>nuclei</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>199 healthy adults (age 18-80+)</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>8 classes / 27 subclasses; 15 subclasses with &gt;=50 nuclei in &gt;=100 donors</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>875,806</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>84ce6837 'Aging_Cohort'</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>Endo/Mural thin (&gt;=50 nuclei in ~80 donors). Arm G possible</t>
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="42.75" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>ALTERNATIVE</t>
@@ -3272,7 +3493,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="28.5" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>
@@ -3349,84 +3570,84 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSED (choose v3 or v2 subset)</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+    <row r="12" ht="42.75" customFormat="1" customHeight="1" s="6">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>PROPOSED: 3' v2 subset</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>training + held-out + E' (by donor)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>colon</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>CRC + adjacent normal</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Pelka 2021, doi:10.1016/j.cell.2021.08.003</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Cell 2021; CELLxGENE 2025-08-05</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>10x 3' v3 (or 3' v2)</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>3' v3: 20 (5 with normal cells); 3' v2: 43 (32 with normal)</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>3' v2: 43 donors, 32 with paired tumour + normal (30 with &gt;=500 cells each); 3' v3: 20 (5 paired)</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>45 (3' v3); all compartments</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>103,511 (v3) / 266,604 (v2)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>PRE</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>4d82bd8e 'All Cells'</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>Epithelium, immune and stroma. Arm G not possible for colon</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>
@@ -3503,7 +3724,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="28.5" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>
@@ -3580,7 +3801,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="28.5" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>
@@ -3657,463 +3878,694 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="28.5" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>ALTERNATIVE</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>training + held-out + E' (by donor)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>CRC (tumour only)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>GEO GSE312983 (CRC across the age continuum, snRNA atlas)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>GEO public 2026-09-23</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>10x 3' (version TO VERIFY)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>nuclei</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>52 (Tier2) / 7 (Tier1); all compartments</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>850,222</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>TO VERIFY</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>GEO h5ad (54 GB)</t>
+        </is>
+      </c>
+      <c r="O16" s="10" t="inlineStr">
+        <is>
+          <t>RAW COUNTS ONLY FOR 4,070 HVGs (layers/counts); all 36,601 genes only log-normalised (raw/X). No normal tissue. FASTQ controlled (dbGaP).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="71.25" customFormat="1" customHeight="1" s="8">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ALTERNATIVE (preferred GEO colon)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>training + held-out + E' (by donor)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>CRC + matched normal</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Lee 2020, GSE132465, doi:10.1038/s41588-020-0636-z</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>GEO 2020-04-04</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>10x 3' (version TO VERIFY)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>23 (10 with normal)</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Cell_type + Cell_subtype</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>63,689</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>TO VERIFY</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>GEO (raw UMI matrix)</t>
+        </is>
+      </c>
+      <c r="O17" s="12" t="inlineStr">
+        <is>
+          <t>PREFERRED over GSE166555 (Claude, 2026-10-23): meets every rule; one raw UMI matrix with all genes; per-cell patient, tumour/normal, cell type and subtype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28.5" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ALTERNATIVE</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>training + held-out + E' (by donor)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>CRC + normal</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Uhlitz 2021, GSE166555, doi:10.15252/emmm.202114123</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>GEO 2021-02-11</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>10x 3' v2</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>per compartment (epi/imm/str)</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>~68,700</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>TO VERIFY</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>GEO (RAW.tar per sample)</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>Second choice after GSE132465: only 12 donors (just above the minimum of 10); raw counts only per sample inside GSE166555_RAW.tar; labels split by compartment (epi/imm/str).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28.5" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ALTERNATIVE (replaced by Wells 2025)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
           <t>training 4 / held-out 1 / E' 1</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>lymphoid (lymph node)</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>normal (organ donors)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Tabula Sapiens v1, doi:10.1126/science.abl4896</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>2022 (CELLxGENE 2021-07)</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>10x 3' v3</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>6 (TSP2, 7, 14, 21, 25, 27; age 45-69)</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>23; 7 with &gt;=50 cells in all 6 donors</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>~79,000 (3' v3 LN cells)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>PRE (in GEM-1 training)</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>e5f58829 'Lymph_Node'</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>Stroma 65 + endothelium 134 cells (dropped by &gt;=50 rule). B cells not subdivided</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="20" ht="28.5" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>TO VERIFY (could replace Tabula Sapiens)</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>training + held-out + E'</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>lymphoid (tonsil)</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>tonsillectomy, children + adults</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>Massoni-Badosa 2024, doi:10.1016/j.immuni.2024.01.006</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Immunity 2024-02-13</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>10x 3' v3.1 (5' v1.1 and multiome also used: per-donor mapping TO VERIFY)</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>cells (cell hashing)</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>up to 17 (6 children, 8 young adults, 3 older adults)</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>121 types/states</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>~377,000</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L20" s="7" t="inlineStr">
         <is>
           <t>PRE</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M20" s="7" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N20" s="7" t="inlineStr">
         <is>
           <t>not on CELLxGENE: HCATonsilData (Bioconductor), Zenodo 10.5281/zenodo.10373041</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="O20" s="7" t="inlineStr">
         <is>
           <t>Check donors per chemistry in HCATonsilData (needs R)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="21" ht="28.5" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>ALTERNATIVE</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>training + held-out + E'</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>lymphoid (lymph node)</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Fergusson 2025, doi:10.1016/j.celrep.2025.115938</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>CELLxGENE 2025-07-08</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>10x 3' v3</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>13 broad</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>186,822</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>POST? TO VERIFY</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>69f13fde</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>T/B cells partly depleted, ILC/NK enriched: not a normal lymph-node mix</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>lymphoid (tonsil)</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>children</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>King 2021, doi:10.1126/sciimmunol.abe6291</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>2021-02-12</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>1 donor 10x 3' v2 + 6 donors 10x 5' v1</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>1 on 3'</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>32,607</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>PRE</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>GRCh38, Cell Ranger 3.0.0</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>3a2af25b</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>Only 1 donor on 3' (rule 3)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>PROPOSED (2026-10-23)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>training + held-out + E' (by donor)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>lymphoid (lymph node)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Wells 2025, doi:10.1038/s41590-025-02241-4</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>bioRxiv 2024-01-03 (data not released: 'will be made available'); GEO GSE299043 + CELLxGENE 2025-06-06</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>10x 5' v2</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>22 (inguinal/mesenteric/thoracic LN; ages 20s-70s)</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>31 (CELLxGENE); 9 with &gt;=50 cells in &gt;=20 donors</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>401,959 (5' v2 LN)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>POST (data first public 2025-06)</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>cc431242</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>Immune cells only: no stroma or endothelium. Most donors have 2-3 LN sites (choose one site or pool per donor: to decide). Replaces Tabula Sapiens (6 donors).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>lymphoid (lymph node)</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Wells 2025, doi:10.1038/s41590-025-02241-4</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>bioRxiv 2024-01-04</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>22 donors 10x 5' v2; 2 on 3' v3</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Xu 2023 / Dominguez Conde 2022</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2022-2023</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>2 on 3'</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>401,959 (5' v2)</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>3' v2: 6; 3' v3: 2 (same 2 donors as Wells)</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>24-31</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>PRE</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>cc431242</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>5' chemistry (rule 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>lymphoid (lymph node)</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Xu 2023 / Dominguez Conde 2022</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>2022-2023</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>cells</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>3' v2: 6; 3' v3: 2 (same 2 donors as Wells)</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>24-31</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>PRE</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>854c0855 / 62ef75e4</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>Mixed chemistries; duplicated donors across atlases</t>
         </is>

</xml_diff>

<commit_message>
T2: DECISIONS add Luca's 2026-10-26 answers; ADEMP v0.1 updated E′, noise ceiling, deconv methods; intro v4 updated deconv methods; letture add Spotless and Li 2023; inventory add GEM-1 cutoff rule
</commit_message>
<xml_diff>
--- a/thesis/data_inventory.xlsx
+++ b/thesis/data_inventory.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-3240" yWindow="-21710" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="selected" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="selected" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -36,18 +36,26 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="FFC00000"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00006100"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
     </font>
     <font>
-      <color rgb="00000000"/>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -118,7 +126,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -126,7 +134,74 @@
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -3260,8 +3335,13 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5. GEM-1 cutoff criterion (DECISIONS 2026-10-26): gem-1-sc was trained on the July 2024 version of CELLxGENE (GEM-1 preprint, Methods). A dataset is post-cutoff if it was NOT in CELLxGENE in July 2024. The column cutoff (GEM-1) below was filled with the first public date and must be rechecked with this criterion. Note: Pelka 2021 appears on CELLxGENE only since 2025-08-05, so it may be post-cutoff for gem-1-sc (to verify).</t>
+        </is>
+      </c>
+    </row>
     <row r="8" ht="28.5" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -4340,7 +4420,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="28.5" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>
@@ -4417,73 +4497,73 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="23" ht="99.75" customFormat="1" customHeight="1" s="6">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>PROPOSED (2026-10-23)</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>training + held-out + E' (by donor)</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>lymphoid (lymph node)</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Wells 2025, doi:10.1038/s41590-025-02241-4</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>bioRxiv 2024-01-03 (data not released: 'will be made available'); GEO GSE299043 + CELLxGENE 2025-06-06</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>10x 5' v2</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>22 (inguinal/mesenteric/thoracic LN; ages 20s-70s)</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>31 (CELLxGENE); 9 with &gt;=50 cells in &gt;=20 donors</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>401,959 (5' v2 LN)</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
         <is>
           <t>POST (data first public 2025-06)</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="M23" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>cc431242</t>
         </is>
@@ -4494,7 +4574,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="28.5" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>REJECTED</t>

</xml_diff>

<commit_message>
T2: DECISIONS refine Dataset row, add cutoff and split rows; ADEMP v0.2 donor counts and noise ceiling; inventory rule 5; Methods v0; 01_download.R
</commit_message>
<xml_diff>
--- a/thesis/data_inventory.xlsx
+++ b/thesis/data_inventory.xlsx
@@ -3338,7 +3338,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5. GEM-1 cutoff criterion (DECISIONS 2026-10-26): gem-1-sc was trained on the July 2024 version of CELLxGENE (GEM-1 preprint, Methods). A dataset is post-cutoff if it was NOT in CELLxGENE in July 2024. The column cutoff (GEM-1) below was filled with the first public date and must be rechecked with this criterion. Note: Pelka 2021 appears on CELLxGENE only since 2025-08-05, so it may be post-cutoff for gem-1-sc (to verify).</t>
+          <t>5. GEM-1 cutoff criterion (DECISIONS 2026-10-27, awaiting Luca): gem-1-sc was trained on the July 2024 version of CELLxGENE (GEM-1 preprint, Methods). A dataset is post-cutoff if its PROCESSED count matrix with cell labels became public after July 2024; raw reads do not count. Both dates (raw / processed) are recorded in 'date (first public)'.</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
     <row r="9" ht="42.75" customFormat="1" customHeight="1" s="6">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>SELECTED (2026-10-26)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>preprint 2024-10-31; CELLxGENE 2025-07-29</t>
+          <t>raw FASTQ 2024-04-22 (AD Knowledge Portal release 24.4); processed h5ad June 2025 (release 25.6); preprint 2024-10-31; CELLxGENE 2025-07-29</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>POST (processed data June 2025; raw reads public before cutoff: declared limit)</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Endo/Mural thin (&gt;=50 nuclei in ~80 donors). Arm G possible</t>
+          <t>Training = all eligible healthy adults except held-out and E' (~198; exact count from 02_split.R; obs also has adolescents and non-normal donors to exclude). Endo/Mural thin (&gt;=50 nuclei in ~80 donors). Arm G possible</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3653,7 @@
     <row r="12" ht="42.75" customFormat="1" customHeight="1" s="6">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>PROPOSED: 3' v2 subset</t>
+          <t>SELECTED (DECISIONS 2026-10-26 "Dataset", refined 2026-10-27, awaiting Luca): 3' v2, MMRp tumours only</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>CRC + adjacent normal</t>
+          <t>CRC, MMRp tumours only (DECISIONS 2026-10-26 "Dataset", refined 2026-10-27, awaiting Luca)</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Cell 2021; CELLxGENE 2025-08-05</t>
+          <t>processed GEO GSE178341 2021-08-26; Cell 2021; CELLxGENE 2025-08-05; raw: not checked</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -3693,7 +3693,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>3' v2: 43 donors, 32 with paired tumour + normal (30 with &gt;=500 cells each); 3' v3: 20 (5 paired)</t>
+          <t>3' v2 MMRp tumours: 20 donors (all &gt;=500 cells); split 18 / 1 / 1. (3' v2 all tumours 43; MMRd 23)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -3703,12 +3703,12 @@
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>103,511 (v3) / 266,604 (v2)</t>
+          <t>89,242 (3' v2 MMRp tumour cells)</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>PRE (processed 2021)</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>Epithelium, immune and stroma. Arm G not possible for colon</t>
+          <t>Epithelium, immune and stroma. MMRd and normal excluded (Pelka 2021: subtypes differ in composition and within-type expression). C130 has 2 lesions (same split). Arm G not possible for colon</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
     <row r="23" ht="99.75" customFormat="1" customHeight="1" s="6">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>PROPOSED (2026-10-23)</t>
+          <t>SELECTED (DECISIONS 2026-10-26 "Dataset", refined 2026-10-27, awaiting Luca): thoracic LN only</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>lymphoid (lymph node)</t>
+          <t>lymphoid (thoracic lymph node)</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -4525,7 +4525,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>bioRxiv 2024-01-03 (data not released: 'will be made available'); GEO GSE299043 + CELLxGENE 2025-06-06</t>
+          <t>processed GEO GSE299043 + CELLxGENE 2025-06-06; bioRxiv 2024-01-03 said data 'will be made available'; raw: not on GEO (not checked)</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>22 (inguinal/mesenteric/thoracic LN; ages 20s-70s)</t>
+          <t>thoracic LN: 21 donors; split 19 / 1 / 1 (all LN sites: 22)</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -4550,12 +4550,12 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>401,959 (5' v2 LN)</t>
+          <t>185,437 (5' v2 thoracic LN cells)</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>POST (data first public 2025-06)</t>
+          <t>POST (processed data 2025-06-06)</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="O23" s="14" t="inlineStr">
         <is>
-          <t>Immune cells only: no stroma or endothelium. Most donors have 2-3 LN sites (choose one site or pool per donor: to decide). Replaces Tabula Sapiens (6 donors).</t>
+          <t>Immune cells only: no stroma or endothelium. Thoracic only (DECISIONS 2026-10-26 "Dataset", refined 2026-10-27, awaiting Luca); inguinal (9 donors) and mesenteric excluded. Donor 778C has 57,317 cells (check B). Replaces Tabula Sapiens.</t>
         </is>
       </c>
     </row>

</xml_diff>